<commit_message>
update scripts with more metrics, add dat-to-csv script
</commit_message>
<xml_diff>
--- a/OpportunityUCIDataset/events.xlsx
+++ b/OpportunityUCIDataset/events.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C218"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,10 +435,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>379.396</v>
+        <v>80.93300000000001</v>
       </c>
       <c r="B2" t="n">
-        <v>380.296</v>
+        <v>82.099</v>
       </c>
       <c r="C2" t="n">
         <v>405</v>
@@ -446,21 +446,21 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>380.363</v>
+        <v>82.133</v>
       </c>
       <c r="B3" t="n">
-        <v>383.23</v>
+        <v>82.699</v>
       </c>
       <c r="C3" t="n">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>390.429</v>
+        <v>87.13200000000001</v>
       </c>
       <c r="B4" t="n">
-        <v>391.263</v>
+        <v>88.29900000000001</v>
       </c>
       <c r="C4" t="n">
         <v>405</v>
@@ -468,43 +468,43 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>392.696</v>
+        <v>88.33199999999999</v>
       </c>
       <c r="B5" t="n">
-        <v>395.029</v>
+        <v>90.79900000000001</v>
       </c>
       <c r="C5" t="n">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>395.696</v>
+        <v>90.83199999999999</v>
       </c>
       <c r="B6" t="n">
-        <v>396.163</v>
+        <v>91.199</v>
       </c>
       <c r="C6" t="n">
-        <v>412</v>
+        <v>403</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>431.029</v>
+        <v>91.232</v>
       </c>
       <c r="B7" t="n">
-        <v>431.496</v>
+        <v>91.899</v>
       </c>
       <c r="C7" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>452.929</v>
+        <v>96.932</v>
       </c>
       <c r="B8" t="n">
-        <v>453.529</v>
+        <v>98.099</v>
       </c>
       <c r="C8" t="n">
         <v>405</v>
@@ -512,76 +512,76 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>453.829</v>
+        <v>98.13200000000001</v>
       </c>
       <c r="B9" t="n">
-        <v>457.029</v>
+        <v>99.79900000000001</v>
       </c>
       <c r="C9" t="n">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>457.062</v>
+        <v>99.83199999999999</v>
       </c>
       <c r="B10" t="n">
-        <v>457.429</v>
+        <v>101.999</v>
       </c>
       <c r="C10" t="n">
-        <v>412</v>
+        <v>404</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>465.395</v>
+        <v>102.032</v>
       </c>
       <c r="B11" t="n">
-        <v>466.062</v>
+        <v>102.699</v>
       </c>
       <c r="C11" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>466.929</v>
+        <v>102.732</v>
       </c>
       <c r="B12" t="n">
-        <v>467.262</v>
+        <v>103.399</v>
       </c>
       <c r="C12" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>473.395</v>
+        <v>103.432</v>
       </c>
       <c r="B13" t="n">
-        <v>473.729</v>
+        <v>106.599</v>
       </c>
       <c r="C13" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>474.829</v>
+        <v>106.632</v>
       </c>
       <c r="B14" t="n">
-        <v>477.062</v>
+        <v>108.699</v>
       </c>
       <c r="C14" t="n">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>477.429</v>
+        <v>108.732</v>
       </c>
       <c r="B15" t="n">
-        <v>477.762</v>
+        <v>108.999</v>
       </c>
       <c r="C15" t="n">
         <v>412</v>
@@ -589,21 +589,21 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>721.093</v>
+        <v>113.832</v>
       </c>
       <c r="B16" t="n">
-        <v>723.193</v>
+        <v>114.399</v>
       </c>
       <c r="C16" t="n">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>723.693</v>
+        <v>114.432</v>
       </c>
       <c r="B17" t="n">
-        <v>725.259</v>
+        <v>117.332</v>
       </c>
       <c r="C17" t="n">
         <v>404</v>
@@ -611,21 +611,21 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>732.926</v>
+        <v>117.365</v>
       </c>
       <c r="B18" t="n">
-        <v>735.059</v>
+        <v>117.632</v>
       </c>
       <c r="C18" t="n">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>735.126</v>
+        <v>117.665</v>
       </c>
       <c r="B19" t="n">
-        <v>735.626</v>
+        <v>118.365</v>
       </c>
       <c r="C19" t="n">
         <v>412</v>
@@ -633,10 +633,10 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>751.359</v>
+        <v>123.532</v>
       </c>
       <c r="B20" t="n">
-        <v>751.792</v>
+        <v>124.399</v>
       </c>
       <c r="C20" t="n">
         <v>405</v>
@@ -644,164 +644,164 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>751.859</v>
+        <v>132.199</v>
       </c>
       <c r="B21" t="n">
-        <v>753.059</v>
+        <v>133.399</v>
       </c>
       <c r="C21" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>753.092</v>
+        <v>133.432</v>
       </c>
       <c r="B22" t="n">
-        <v>754.259</v>
+        <v>135.265</v>
       </c>
       <c r="C22" t="n">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>755.026</v>
+        <v>136.032</v>
       </c>
       <c r="B23" t="n">
-        <v>755.4589999999999</v>
+        <v>138.399</v>
       </c>
       <c r="C23" t="n">
-        <v>412</v>
+        <v>404</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>761.526</v>
+        <v>138.432</v>
       </c>
       <c r="B24" t="n">
-        <v>763.659</v>
+        <v>139.199</v>
       </c>
       <c r="C24" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>763.692</v>
+        <v>144.932</v>
       </c>
       <c r="B25" t="n">
-        <v>769.792</v>
+        <v>145.532</v>
       </c>
       <c r="C25" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>769.826</v>
+        <v>145.565</v>
       </c>
       <c r="B26" t="n">
-        <v>770.4589999999999</v>
+        <v>146.365</v>
       </c>
       <c r="C26" t="n">
-        <v>412</v>
+        <v>401</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>771.992</v>
+        <v>146.399</v>
       </c>
       <c r="B27" t="n">
-        <v>772.4589999999999</v>
+        <v>148.599</v>
       </c>
       <c r="C27" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>772.8920000000001</v>
+        <v>148.632</v>
       </c>
       <c r="B28" t="n">
-        <v>773.492</v>
+        <v>149.599</v>
       </c>
       <c r="C28" t="n">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>773.559</v>
+        <v>155.132</v>
       </c>
       <c r="B29" t="n">
-        <v>773.792</v>
+        <v>155.632</v>
       </c>
       <c r="C29" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>780.4589999999999</v>
+        <v>156.498</v>
       </c>
       <c r="B30" t="n">
-        <v>781.059</v>
+        <v>156.898</v>
       </c>
       <c r="C30" t="n">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>781.126</v>
+        <v>157.232</v>
       </c>
       <c r="B31" t="n">
-        <v>784.992</v>
+        <v>160.098</v>
       </c>
       <c r="C31" t="n">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>785.625</v>
+        <v>160.132</v>
       </c>
       <c r="B32" t="n">
-        <v>786.8920000000001</v>
+        <v>161.565</v>
       </c>
       <c r="C32" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>787.025</v>
+        <v>315.73</v>
       </c>
       <c r="B33" t="n">
-        <v>788.825</v>
+        <v>317.397</v>
       </c>
       <c r="C33" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>788.925</v>
+        <v>317.43</v>
       </c>
       <c r="B34" t="n">
-        <v>789.259</v>
+        <v>320.197</v>
       </c>
       <c r="C34" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>789.325</v>
+        <v>320.23</v>
       </c>
       <c r="B35" t="n">
-        <v>789.759</v>
+        <v>321.497</v>
       </c>
       <c r="C35" t="n">
         <v>405</v>
@@ -809,10 +809,10 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>789.859</v>
+        <v>321.53</v>
       </c>
       <c r="B36" t="n">
-        <v>800.525</v>
+        <v>325.597</v>
       </c>
       <c r="C36" t="n">
         <v>413</v>
@@ -820,10 +820,10 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>801.025</v>
+        <v>325.63</v>
       </c>
       <c r="B37" t="n">
-        <v>801.425</v>
+        <v>326.23</v>
       </c>
       <c r="C37" t="n">
         <v>412</v>
@@ -831,10 +831,10 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>869.225</v>
+        <v>328.23</v>
       </c>
       <c r="B38" t="n">
-        <v>870.191</v>
+        <v>329.197</v>
       </c>
       <c r="C38" t="n">
         <v>405</v>
@@ -842,65 +842,65 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>875.625</v>
+        <v>329.23</v>
       </c>
       <c r="B39" t="n">
-        <v>875.891</v>
+        <v>329.43</v>
       </c>
       <c r="C39" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>875.925</v>
+        <v>330.63</v>
       </c>
       <c r="B40" t="n">
-        <v>877.591</v>
+        <v>332.897</v>
       </c>
       <c r="C40" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>877.625</v>
+        <v>332.93</v>
       </c>
       <c r="B41" t="n">
-        <v>878.458</v>
+        <v>337.697</v>
       </c>
       <c r="C41" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>882.491</v>
+        <v>337.73</v>
       </c>
       <c r="B42" t="n">
-        <v>893.2910000000001</v>
+        <v>337.997</v>
       </c>
       <c r="C42" t="n">
-        <v>402</v>
+        <v>412</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>895.158</v>
+        <v>338.03</v>
       </c>
       <c r="B43" t="n">
-        <v>896.158</v>
+        <v>338.597</v>
       </c>
       <c r="C43" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>897.091</v>
+        <v>338.63</v>
       </c>
       <c r="B44" t="n">
-        <v>899.391</v>
+        <v>340.097</v>
       </c>
       <c r="C44" t="n">
         <v>413</v>
@@ -908,32 +908,32 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>901.224</v>
+        <v>340.13</v>
       </c>
       <c r="B45" t="n">
-        <v>901.824</v>
+        <v>340.697</v>
       </c>
       <c r="C45" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>902.8579999999999</v>
+        <v>340.73</v>
       </c>
       <c r="B46" t="n">
-        <v>904.258</v>
+        <v>341.197</v>
       </c>
       <c r="C46" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>905.191</v>
+        <v>341.23</v>
       </c>
       <c r="B47" t="n">
-        <v>905.891</v>
+        <v>342.897</v>
       </c>
       <c r="C47" t="n">
         <v>413</v>
@@ -941,65 +941,65 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>908.724</v>
+        <v>342.93</v>
       </c>
       <c r="B48" t="n">
-        <v>909.524</v>
+        <v>345.897</v>
       </c>
       <c r="C48" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>909.591</v>
+        <v>411.129</v>
       </c>
       <c r="B49" t="n">
-        <v>910.924</v>
+        <v>411.929</v>
       </c>
       <c r="C49" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>911.8579999999999</v>
+        <v>411.963</v>
       </c>
       <c r="B50" t="n">
-        <v>913.391</v>
+        <v>416.096</v>
       </c>
       <c r="C50" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>913.424</v>
+        <v>416.129</v>
       </c>
       <c r="B51" t="n">
-        <v>914.424</v>
+        <v>416.996</v>
       </c>
       <c r="C51" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>914.491</v>
+        <v>421.629</v>
       </c>
       <c r="B52" t="n">
-        <v>916.658</v>
+        <v>422.162</v>
       </c>
       <c r="C52" t="n">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>916.724</v>
+        <v>422.196</v>
       </c>
       <c r="B53" t="n">
-        <v>918.557</v>
+        <v>430.562</v>
       </c>
       <c r="C53" t="n">
         <v>413</v>
@@ -1007,175 +1007,175 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>918.624</v>
+        <v>431.096</v>
       </c>
       <c r="B54" t="n">
-        <v>919.891</v>
+        <v>432.096</v>
       </c>
       <c r="C54" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>923.224</v>
+        <v>432.129</v>
       </c>
       <c r="B55" t="n">
-        <v>924.2910000000001</v>
+        <v>438.696</v>
       </c>
       <c r="C55" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>924.324</v>
+        <v>438.729</v>
       </c>
       <c r="B56" t="n">
-        <v>925.7569999999999</v>
+        <v>442.162</v>
       </c>
       <c r="C56" t="n">
-        <v>413</v>
+        <v>402</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>925.7910000000001</v>
+        <v>442.196</v>
       </c>
       <c r="B57" t="n">
-        <v>927.991</v>
+        <v>445.096</v>
       </c>
       <c r="C57" t="n">
-        <v>407</v>
+        <v>413</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>928.024</v>
+        <v>445.329</v>
       </c>
       <c r="B58" t="n">
-        <v>929.2569999999999</v>
+        <v>446.029</v>
       </c>
       <c r="C58" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>929.2910000000001</v>
+        <v>446.096</v>
       </c>
       <c r="B59" t="n">
-        <v>929.824</v>
+        <v>447.596</v>
       </c>
       <c r="C59" t="n">
-        <v>407</v>
+        <v>413</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>929.891</v>
+        <v>447.629</v>
       </c>
       <c r="B60" t="n">
-        <v>931.2910000000001</v>
+        <v>449.396</v>
       </c>
       <c r="C60" t="n">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>931.724</v>
+        <v>449.429</v>
       </c>
       <c r="B61" t="n">
-        <v>932.391</v>
+        <v>451.295</v>
       </c>
       <c r="C61" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>934.691</v>
+        <v>451.329</v>
       </c>
       <c r="B62" t="n">
-        <v>935.2910000000001</v>
+        <v>451.795</v>
       </c>
       <c r="C62" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>936.124</v>
+        <v>454.929</v>
       </c>
       <c r="B63" t="n">
-        <v>937.391</v>
+        <v>455.795</v>
       </c>
       <c r="C63" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>937.424</v>
+        <v>455.829</v>
       </c>
       <c r="B64" t="n">
-        <v>941.357</v>
+        <v>457.362</v>
       </c>
       <c r="C64" t="n">
-        <v>407</v>
+        <v>413</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>941.424</v>
+        <v>457.395</v>
       </c>
       <c r="B65" t="n">
-        <v>943.891</v>
+        <v>458.695</v>
       </c>
       <c r="C65" t="n">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>943.924</v>
+        <v>458.729</v>
       </c>
       <c r="B66" t="n">
-        <v>944.2910000000001</v>
+        <v>460.162</v>
       </c>
       <c r="C66" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>947.124</v>
+        <v>460.229</v>
       </c>
       <c r="B67" t="n">
-        <v>948.691</v>
+        <v>460.895</v>
       </c>
       <c r="C67" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>949.324</v>
+        <v>462.929</v>
       </c>
       <c r="B68" t="n">
-        <v>952.89</v>
+        <v>464.029</v>
       </c>
       <c r="C68" t="n">
-        <v>402</v>
+        <v>405</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>955.924</v>
+        <v>464.062</v>
       </c>
       <c r="B69" t="n">
-        <v>957.157</v>
+        <v>465.362</v>
       </c>
       <c r="C69" t="n">
         <v>413</v>
@@ -1183,54 +1183,54 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>957.824</v>
+        <v>465.395</v>
       </c>
       <c r="B70" t="n">
-        <v>958.59</v>
+        <v>467.962</v>
       </c>
       <c r="C70" t="n">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>961.824</v>
+        <v>467.995</v>
       </c>
       <c r="B71" t="n">
-        <v>962.2569999999999</v>
+        <v>469.562</v>
       </c>
       <c r="C71" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>963.224</v>
+        <v>469.595</v>
       </c>
       <c r="B72" t="n">
-        <v>966.657</v>
+        <v>470.395</v>
       </c>
       <c r="C72" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>966.6900000000001</v>
+        <v>471.629</v>
       </c>
       <c r="B73" t="n">
-        <v>968.824</v>
+        <v>472.595</v>
       </c>
       <c r="C73" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>969.6900000000001</v>
+        <v>472.629</v>
       </c>
       <c r="B74" t="n">
-        <v>970.224</v>
+        <v>473.795</v>
       </c>
       <c r="C74" t="n">
         <v>413</v>
@@ -1238,21 +1238,21 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>971.724</v>
+        <v>473.829</v>
       </c>
       <c r="B75" t="n">
-        <v>972.557</v>
+        <v>475.995</v>
       </c>
       <c r="C75" t="n">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>1003.123</v>
+        <v>476.029</v>
       </c>
       <c r="B76" t="n">
-        <v>1013.29</v>
+        <v>478.062</v>
       </c>
       <c r="C76" t="n">
         <v>413</v>
@@ -1260,10 +1260,10 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>1068.923</v>
+        <v>480.329</v>
       </c>
       <c r="B77" t="n">
-        <v>1069.589</v>
+        <v>481.095</v>
       </c>
       <c r="C77" t="n">
         <v>405</v>
@@ -1271,10 +1271,10 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>1069.623</v>
+        <v>481.129</v>
       </c>
       <c r="B78" t="n">
-        <v>1070.589</v>
+        <v>482.362</v>
       </c>
       <c r="C78" t="n">
         <v>413</v>
@@ -1282,43 +1282,43 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1071.623</v>
+        <v>482.429</v>
       </c>
       <c r="B79" t="n">
-        <v>1072.289</v>
+        <v>484.162</v>
       </c>
       <c r="C79" t="n">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>1072.389</v>
+        <v>484.195</v>
       </c>
       <c r="B80" t="n">
-        <v>1073.189</v>
+        <v>485.495</v>
       </c>
       <c r="C80" t="n">
-        <v>404</v>
+        <v>413</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>1074.323</v>
+        <v>485.528</v>
       </c>
       <c r="B81" t="n">
-        <v>1075.123</v>
+        <v>486.495</v>
       </c>
       <c r="C81" t="n">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>1075.523</v>
+        <v>488.528</v>
       </c>
       <c r="B82" t="n">
-        <v>1075.923</v>
+        <v>489.195</v>
       </c>
       <c r="C82" t="n">
         <v>405</v>
@@ -1326,10 +1326,10 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>1075.956</v>
+        <v>489.228</v>
       </c>
       <c r="B83" t="n">
-        <v>1077.323</v>
+        <v>490.395</v>
       </c>
       <c r="C83" t="n">
         <v>413</v>
@@ -1337,76 +1337,76 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1077.389</v>
+        <v>490.428</v>
       </c>
       <c r="B84" t="n">
-        <v>1077.689</v>
+        <v>491.895</v>
       </c>
       <c r="C84" t="n">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1077.723</v>
+        <v>491.928</v>
       </c>
       <c r="B85" t="n">
-        <v>1078.989</v>
+        <v>492.962</v>
       </c>
       <c r="C85" t="n">
-        <v>404</v>
+        <v>413</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>1079.023</v>
+        <v>493.028</v>
       </c>
       <c r="B86" t="n">
-        <v>1079.556</v>
+        <v>493.995</v>
       </c>
       <c r="C86" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>1086.122</v>
+        <v>494.928</v>
       </c>
       <c r="B87" t="n">
-        <v>1086.989</v>
+        <v>495.695</v>
       </c>
       <c r="C87" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>1087.056</v>
+        <v>495.728</v>
       </c>
       <c r="B88" t="n">
-        <v>1087.589</v>
+        <v>496.695</v>
       </c>
       <c r="C88" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>1088.356</v>
+        <v>496.728</v>
       </c>
       <c r="B89" t="n">
-        <v>1088.622</v>
+        <v>497.662</v>
       </c>
       <c r="C89" t="n">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>1088.722</v>
+        <v>497.695</v>
       </c>
       <c r="B90" t="n">
-        <v>1089.989</v>
+        <v>498.895</v>
       </c>
       <c r="C90" t="n">
         <v>413</v>
@@ -1414,10 +1414,10 @@
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>1090.489</v>
+        <v>498.928</v>
       </c>
       <c r="B91" t="n">
-        <v>1091.422</v>
+        <v>499.495</v>
       </c>
       <c r="C91" t="n">
         <v>412</v>
@@ -1425,10 +1425,10 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1103.722</v>
+        <v>501.128</v>
       </c>
       <c r="B92" t="n">
-        <v>1105.156</v>
+        <v>501.562</v>
       </c>
       <c r="C92" t="n">
         <v>405</v>
@@ -1436,10 +1436,10 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>1105.422</v>
+        <v>501.595</v>
       </c>
       <c r="B93" t="n">
-        <v>1109.256</v>
+        <v>504.095</v>
       </c>
       <c r="C93" t="n">
         <v>413</v>
@@ -1447,43 +1447,43 @@
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>1109.356</v>
+        <v>504.128</v>
       </c>
       <c r="B94" t="n">
-        <v>1109.989</v>
+        <v>505.128</v>
       </c>
       <c r="C94" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>1115.822</v>
+        <v>505.162</v>
       </c>
       <c r="B95" t="n">
-        <v>1117.055</v>
+        <v>508.562</v>
       </c>
       <c r="C95" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>1117.089</v>
+        <v>508.595</v>
       </c>
       <c r="B96" t="n">
-        <v>1122.422</v>
+        <v>510.095</v>
       </c>
       <c r="C96" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>1137.222</v>
+        <v>515.662</v>
       </c>
       <c r="B97" t="n">
-        <v>1137.889</v>
+        <v>517.061</v>
       </c>
       <c r="C97" t="n">
         <v>405</v>
@@ -1491,219 +1491,219 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>1138.555</v>
+        <v>517.095</v>
       </c>
       <c r="B98" t="n">
-        <v>1139.389</v>
+        <v>517.795</v>
       </c>
       <c r="C98" t="n">
-        <v>406</v>
+        <v>401</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>1139.789</v>
+        <v>517.828</v>
       </c>
       <c r="B99" t="n">
-        <v>1140.422</v>
+        <v>518.595</v>
       </c>
       <c r="C99" t="n">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>1140.955</v>
+        <v>518.628</v>
       </c>
       <c r="B100" t="n">
-        <v>1141.889</v>
+        <v>519.895</v>
       </c>
       <c r="C100" t="n">
-        <v>413</v>
+        <v>404</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>1142.389</v>
+        <v>519.928</v>
       </c>
       <c r="B101" t="n">
-        <v>1142.889</v>
+        <v>520.295</v>
       </c>
       <c r="C101" t="n">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1142.955</v>
+        <v>520.328</v>
       </c>
       <c r="B102" t="n">
-        <v>1143.989</v>
+        <v>520.895</v>
       </c>
       <c r="C102" t="n">
-        <v>404</v>
+        <v>412</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>1144.022</v>
+        <v>524.761</v>
       </c>
       <c r="B103" t="n">
-        <v>1144.489</v>
+        <v>526.395</v>
       </c>
       <c r="C103" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>1151.222</v>
+        <v>526.428</v>
       </c>
       <c r="B104" t="n">
-        <v>1154.722</v>
+        <v>527.6950000000001</v>
       </c>
       <c r="C104" t="n">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1173.222</v>
+        <v>527.728</v>
       </c>
       <c r="B105" t="n">
-        <v>1176.255</v>
+        <v>527.895</v>
       </c>
       <c r="C105" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>1176.322</v>
+        <v>527.928</v>
       </c>
       <c r="B106" t="n">
-        <v>1177.322</v>
+        <v>529.295</v>
       </c>
       <c r="C106" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>1182.722</v>
+        <v>529.328</v>
       </c>
       <c r="B107" t="n">
-        <v>1182.988</v>
+        <v>530.1609999999999</v>
       </c>
       <c r="C107" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>1184.521</v>
+        <v>530.828</v>
       </c>
       <c r="B108" t="n">
-        <v>1196.955</v>
+        <v>531.1950000000001</v>
       </c>
       <c r="C108" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>1197.021</v>
+        <v>531.228</v>
       </c>
       <c r="B109" t="n">
-        <v>1199.255</v>
+        <v>532.361</v>
       </c>
       <c r="C109" t="n">
-        <v>411</v>
+        <v>404</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>1202.421</v>
+        <v>532.395</v>
       </c>
       <c r="B110" t="n">
-        <v>1203.288</v>
+        <v>533.261</v>
       </c>
       <c r="C110" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>1203.321</v>
+        <v>533.328</v>
       </c>
       <c r="B111" t="n">
-        <v>1203.855</v>
+        <v>533.795</v>
       </c>
       <c r="C111" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>1212.721</v>
+        <v>533.828</v>
       </c>
       <c r="B112" t="n">
-        <v>1213.088</v>
+        <v>535.095</v>
       </c>
       <c r="C112" t="n">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>1213.121</v>
+        <v>535.128</v>
       </c>
       <c r="B113" t="n">
-        <v>1213.688</v>
+        <v>535.595</v>
       </c>
       <c r="C113" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>1217.521</v>
+        <v>535.628</v>
       </c>
       <c r="B114" t="n">
-        <v>1253.354</v>
+        <v>537.095</v>
       </c>
       <c r="C114" t="n">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>1256.354</v>
+        <v>537.128</v>
       </c>
       <c r="B115" t="n">
-        <v>1257.254</v>
+        <v>538.395</v>
       </c>
       <c r="C115" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>1257.321</v>
+        <v>538.428</v>
       </c>
       <c r="B116" t="n">
-        <v>1260.021</v>
+        <v>539.295</v>
       </c>
       <c r="C116" t="n">
-        <v>409</v>
+        <v>404</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>1260.787</v>
+        <v>539.328</v>
       </c>
       <c r="B117" t="n">
-        <v>1262.054</v>
+        <v>540.395</v>
       </c>
       <c r="C117" t="n">
         <v>413</v>
@@ -1711,21 +1711,21 @@
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>1267.021</v>
+        <v>540.428</v>
       </c>
       <c r="B118" t="n">
-        <v>1268.654</v>
+        <v>541.061</v>
       </c>
       <c r="C118" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>1271.121</v>
+        <v>541.095</v>
       </c>
       <c r="B119" t="n">
-        <v>1272.787</v>
+        <v>546.1950000000001</v>
       </c>
       <c r="C119" t="n">
         <v>413</v>
@@ -1733,65 +1733,65 @@
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>1272.854</v>
+        <v>546.228</v>
       </c>
       <c r="B120" t="n">
-        <v>1273.687</v>
+        <v>546.495</v>
       </c>
       <c r="C120" t="n">
-        <v>407</v>
+        <v>412</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>1273.721</v>
+        <v>547.428</v>
       </c>
       <c r="B121" t="n">
-        <v>1274.987</v>
+        <v>548.495</v>
       </c>
       <c r="C121" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>1275.021</v>
+        <v>550.794</v>
       </c>
       <c r="B122" t="n">
-        <v>1275.487</v>
+        <v>551.5940000000001</v>
       </c>
       <c r="C122" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>1275.721</v>
+        <v>551.628</v>
       </c>
       <c r="B123" t="n">
-        <v>1276.987</v>
+        <v>552.361</v>
       </c>
       <c r="C123" t="n">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>1278.854</v>
+        <v>552.694</v>
       </c>
       <c r="B124" t="n">
-        <v>1279.587</v>
+        <v>555.0940000000001</v>
       </c>
       <c r="C124" t="n">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>1279.621</v>
+        <v>555.128</v>
       </c>
       <c r="B125" t="n">
-        <v>1280.054</v>
+        <v>562.194</v>
       </c>
       <c r="C125" t="n">
         <v>413</v>
@@ -1799,21 +1799,21 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>1295.654</v>
+        <v>562.228</v>
       </c>
       <c r="B126" t="n">
-        <v>1296.987</v>
+        <v>562.761</v>
       </c>
       <c r="C126" t="n">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>1308.754</v>
+        <v>562.794</v>
       </c>
       <c r="B127" t="n">
-        <v>1310.32</v>
+        <v>563.028</v>
       </c>
       <c r="C127" t="n">
         <v>405</v>
@@ -1821,32 +1821,32 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>1310.387</v>
+        <v>563.061</v>
       </c>
       <c r="B128" t="n">
-        <v>1312.02</v>
+        <v>563.694</v>
       </c>
       <c r="C128" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>1312.087</v>
+        <v>566.228</v>
       </c>
       <c r="B129" t="n">
-        <v>1313.82</v>
+        <v>567.894</v>
       </c>
       <c r="C129" t="n">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>1313.854</v>
+        <v>567.928</v>
       </c>
       <c r="B130" t="n">
-        <v>1315.187</v>
+        <v>570.461</v>
       </c>
       <c r="C130" t="n">
         <v>413</v>
@@ -1854,241 +1854,241 @@
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>1330.92</v>
+        <v>570.5940000000001</v>
       </c>
       <c r="B131" t="n">
-        <v>1332.12</v>
+        <v>572.494</v>
       </c>
       <c r="C131" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>1332.153</v>
+        <v>572.528</v>
       </c>
       <c r="B132" t="n">
-        <v>1334.287</v>
+        <v>573.361</v>
       </c>
       <c r="C132" t="n">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>1334.42</v>
+        <v>573.394</v>
       </c>
       <c r="B133" t="n">
-        <v>1335.153</v>
+        <v>574.494</v>
       </c>
       <c r="C133" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>1336.62</v>
+        <v>574.528</v>
       </c>
       <c r="B134" t="n">
-        <v>1338.353</v>
+        <v>576.394</v>
       </c>
       <c r="C134" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>1338.42</v>
+        <v>576.428</v>
       </c>
       <c r="B135" t="n">
-        <v>1339.753</v>
+        <v>576.894</v>
       </c>
       <c r="C135" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>1339.787</v>
+        <v>576.928</v>
       </c>
       <c r="B136" t="n">
-        <v>1341.653</v>
+        <v>578.328</v>
       </c>
       <c r="C136" t="n">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>1341.82</v>
+        <v>578.361</v>
       </c>
       <c r="B137" t="n">
-        <v>1343.253</v>
+        <v>578.861</v>
       </c>
       <c r="C137" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>1343.32</v>
+        <v>578.894</v>
       </c>
       <c r="B138" t="n">
-        <v>1344.42</v>
+        <v>582.894</v>
       </c>
       <c r="C138" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>1353.153</v>
+        <v>582.928</v>
       </c>
       <c r="B139" t="n">
-        <v>1354.42</v>
+        <v>583.294</v>
       </c>
       <c r="C139" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>1354.453</v>
+        <v>589.261</v>
       </c>
       <c r="B140" t="n">
-        <v>1355.286</v>
+        <v>591.1609999999999</v>
       </c>
       <c r="C140" t="n">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>1355.32</v>
+        <v>593.227</v>
       </c>
       <c r="B141" t="n">
-        <v>1356.42</v>
+        <v>595.1609999999999</v>
       </c>
       <c r="C141" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>1357.02</v>
+        <v>595.227</v>
       </c>
       <c r="B142" t="n">
-        <v>1358.386</v>
+        <v>595.894</v>
       </c>
       <c r="C142" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>1358.453</v>
+        <v>595.927</v>
       </c>
       <c r="B143" t="n">
-        <v>1359.82</v>
+        <v>597.0940000000001</v>
       </c>
       <c r="C143" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>1359.853</v>
+        <v>597.127</v>
       </c>
       <c r="B144" t="n">
-        <v>1361.82</v>
+        <v>597.494</v>
       </c>
       <c r="C144" t="n">
-        <v>407</v>
+        <v>413</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>1361.853</v>
+        <v>597.527</v>
       </c>
       <c r="B145" t="n">
-        <v>1363.353</v>
+        <v>598.0940000000001</v>
       </c>
       <c r="C145" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>1363.42</v>
+        <v>598.127</v>
       </c>
       <c r="B146" t="n">
-        <v>1364.253</v>
+        <v>599.561</v>
       </c>
       <c r="C146" t="n">
-        <v>412</v>
+        <v>404</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>1368.853</v>
+        <v>599.5940000000001</v>
       </c>
       <c r="B147" t="n">
-        <v>1369.653</v>
+        <v>600.127</v>
       </c>
       <c r="C147" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>1369.72</v>
+        <v>600.1609999999999</v>
       </c>
       <c r="B148" t="n">
-        <v>1371.953</v>
+        <v>602.694</v>
       </c>
       <c r="C148" t="n">
-        <v>409</v>
+        <v>413</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>1372.053</v>
+        <v>611.427</v>
       </c>
       <c r="B149" t="n">
-        <v>1374.053</v>
+        <v>612.361</v>
       </c>
       <c r="C149" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>1374.12</v>
+        <v>612.394</v>
       </c>
       <c r="B150" t="n">
-        <v>1374.686</v>
+        <v>613.227</v>
       </c>
       <c r="C150" t="n">
-        <v>409</v>
+        <v>401</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>1374.72</v>
+        <v>613.261</v>
       </c>
       <c r="B151" t="n">
-        <v>1375.286</v>
+        <v>616.227</v>
       </c>
       <c r="C151" t="n">
-        <v>413</v>
+        <v>406</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>1375.353</v>
+        <v>616.261</v>
       </c>
       <c r="B152" t="n">
-        <v>1375.953</v>
+        <v>616.794</v>
       </c>
       <c r="C152" t="n">
         <v>412</v>
@@ -2096,10 +2096,10 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>1375.986</v>
+        <v>621.994</v>
       </c>
       <c r="B153" t="n">
-        <v>1376.42</v>
+        <v>623.46</v>
       </c>
       <c r="C153" t="n">
         <v>405</v>
@@ -2107,10 +2107,10 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>1376.486</v>
+        <v>623.527</v>
       </c>
       <c r="B154" t="n">
-        <v>1377.653</v>
+        <v>633.194</v>
       </c>
       <c r="C154" t="n">
         <v>413</v>
@@ -2118,32 +2118,32 @@
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>1377.72</v>
+        <v>654.427</v>
       </c>
       <c r="B155" t="n">
-        <v>1379.486</v>
+        <v>664.36</v>
       </c>
       <c r="C155" t="n">
-        <v>407</v>
+        <v>413</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>1381.42</v>
+        <v>664.627</v>
       </c>
       <c r="B156" t="n">
-        <v>1385.153</v>
+        <v>665.693</v>
       </c>
       <c r="C156" t="n">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>1385.219</v>
+        <v>665.727</v>
       </c>
       <c r="B157" t="n">
-        <v>1386.453</v>
+        <v>666.76</v>
       </c>
       <c r="C157" t="n">
         <v>413</v>
@@ -2151,54 +2151,54 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>1386.486</v>
+        <v>666.827</v>
       </c>
       <c r="B158" t="n">
-        <v>1387.286</v>
+        <v>667.9930000000001</v>
       </c>
       <c r="C158" t="n">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>1387.919</v>
+        <v>668.027</v>
       </c>
       <c r="B159" t="n">
-        <v>1388.353</v>
+        <v>669.86</v>
       </c>
       <c r="C159" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>1388.419</v>
+        <v>669.927</v>
       </c>
       <c r="B160" t="n">
-        <v>1389.886</v>
+        <v>670.393</v>
       </c>
       <c r="C160" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>1390.919</v>
+        <v>673.227</v>
       </c>
       <c r="B161" t="n">
-        <v>1391.886</v>
+        <v>673.9930000000001</v>
       </c>
       <c r="C161" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>1395.719</v>
+        <v>675.593</v>
       </c>
       <c r="B162" t="n">
-        <v>1396.586</v>
+        <v>676.593</v>
       </c>
       <c r="C162" t="n">
         <v>405</v>
@@ -2206,131 +2206,131 @@
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>1397.319</v>
+        <v>676.627</v>
       </c>
       <c r="B163" t="n">
-        <v>1398.319</v>
+        <v>680.593</v>
       </c>
       <c r="C163" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>1398.353</v>
+        <v>680.627</v>
       </c>
       <c r="B164" t="n">
-        <v>1401.386</v>
+        <v>683.46</v>
       </c>
       <c r="C164" t="n">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>1401.453</v>
+        <v>683.4930000000001</v>
       </c>
       <c r="B165" t="n">
-        <v>1401.886</v>
+        <v>684.76</v>
       </c>
       <c r="C165" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>1401.919</v>
+        <v>684.793</v>
       </c>
       <c r="B166" t="n">
-        <v>1403.253</v>
+        <v>685.293</v>
       </c>
       <c r="C166" t="n">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>1403.919</v>
+        <v>685.426</v>
       </c>
       <c r="B167" t="n">
-        <v>1406.286</v>
+        <v>686.96</v>
       </c>
       <c r="C167" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>1408.853</v>
+        <v>686.9930000000001</v>
       </c>
       <c r="B168" t="n">
-        <v>1409.886</v>
+        <v>688.093</v>
       </c>
       <c r="C168" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>1421.919</v>
+        <v>688.126</v>
       </c>
       <c r="B169" t="n">
-        <v>1422.719</v>
+        <v>688.393</v>
       </c>
       <c r="C169" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>1422.752</v>
+        <v>689.426</v>
       </c>
       <c r="B170" t="n">
-        <v>1423.552</v>
+        <v>690.426</v>
       </c>
       <c r="C170" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>1426.919</v>
+        <v>690.4930000000001</v>
       </c>
       <c r="B171" t="n">
-        <v>1427.519</v>
+        <v>695.426</v>
       </c>
       <c r="C171" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>1428.052</v>
+        <v>695.46</v>
       </c>
       <c r="B172" t="n">
-        <v>1429.819</v>
+        <v>696.193</v>
       </c>
       <c r="C172" t="n">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>1429.886</v>
+        <v>696.226</v>
       </c>
       <c r="B173" t="n">
-        <v>1430.186</v>
+        <v>696.693</v>
       </c>
       <c r="C173" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>1432.819</v>
+        <v>696.726</v>
       </c>
       <c r="B174" t="n">
-        <v>1434.486</v>
+        <v>697.893</v>
       </c>
       <c r="C174" t="n">
         <v>413</v>
@@ -2338,21 +2338,21 @@
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>1434.519</v>
+        <v>697.926</v>
       </c>
       <c r="B175" t="n">
-        <v>1435.086</v>
+        <v>708.16</v>
       </c>
       <c r="C175" t="n">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>1438.219</v>
+        <v>708.226</v>
       </c>
       <c r="B176" t="n">
-        <v>1440.786</v>
+        <v>716.726</v>
       </c>
       <c r="C176" t="n">
         <v>413</v>
@@ -2360,10 +2360,10 @@
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>1440.819</v>
+        <v>716.793</v>
       </c>
       <c r="B177" t="n">
-        <v>1441.352</v>
+        <v>717.159</v>
       </c>
       <c r="C177" t="n">
         <v>412</v>
@@ -2371,10 +2371,10 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>1443.419</v>
+        <v>717.526</v>
       </c>
       <c r="B178" t="n">
-        <v>1443.986</v>
+        <v>719.193</v>
       </c>
       <c r="C178" t="n">
         <v>405</v>
@@ -2382,10 +2382,10 @@
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>1444.019</v>
+        <v>719.226</v>
       </c>
       <c r="B179" t="n">
-        <v>1444.586</v>
+        <v>720.9930000000001</v>
       </c>
       <c r="C179" t="n">
         <v>413</v>
@@ -2393,21 +2393,21 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>1444.719</v>
+        <v>721.026</v>
       </c>
       <c r="B180" t="n">
-        <v>1445.586</v>
+        <v>723.393</v>
       </c>
       <c r="C180" t="n">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>1445.619</v>
+        <v>723.426</v>
       </c>
       <c r="B181" t="n">
-        <v>1449.086</v>
+        <v>725.326</v>
       </c>
       <c r="C181" t="n">
         <v>413</v>
@@ -2415,175 +2415,175 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>1450.019</v>
+        <v>725.359</v>
       </c>
       <c r="B182" t="n">
-        <v>1452.285</v>
+        <v>725.893</v>
       </c>
       <c r="C182" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>1452.319</v>
+        <v>725.926</v>
       </c>
       <c r="B183" t="n">
-        <v>1453.119</v>
+        <v>727.093</v>
       </c>
       <c r="C183" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>1462.919</v>
+        <v>727.126</v>
       </c>
       <c r="B184" t="n">
-        <v>1463.552</v>
+        <v>728.4589999999999</v>
       </c>
       <c r="C184" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>1463.619</v>
+        <v>728.4930000000001</v>
       </c>
       <c r="B185" t="n">
-        <v>1464.185</v>
+        <v>730.759</v>
       </c>
       <c r="C185" t="n">
-        <v>413</v>
+        <v>407</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>1464.219</v>
+        <v>730.793</v>
       </c>
       <c r="B186" t="n">
-        <v>1464.585</v>
+        <v>732.4589999999999</v>
       </c>
       <c r="C186" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>1465.585</v>
+        <v>732.4930000000001</v>
       </c>
       <c r="B187" t="n">
-        <v>1468.352</v>
+        <v>733.4930000000001</v>
       </c>
       <c r="C187" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>1468.419</v>
+        <v>737.893</v>
       </c>
       <c r="B188" t="n">
-        <v>1470.352</v>
+        <v>738.693</v>
       </c>
       <c r="C188" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>1471.419</v>
+        <v>738.726</v>
       </c>
       <c r="B189" t="n">
-        <v>1471.952</v>
+        <v>740.293</v>
       </c>
       <c r="C189" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>1472.185</v>
+        <v>740.326</v>
       </c>
       <c r="B190" t="n">
-        <v>1474.019</v>
+        <v>741.4930000000001</v>
       </c>
       <c r="C190" t="n">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>1474.619</v>
+        <v>741.526</v>
       </c>
       <c r="B191" t="n">
-        <v>1474.952</v>
+        <v>742.526</v>
       </c>
       <c r="C191" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>1480.219</v>
+        <v>742.559</v>
       </c>
       <c r="B192" t="n">
-        <v>1480.685</v>
+        <v>743.759</v>
       </c>
       <c r="C192" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>1480.719</v>
+        <v>745.026</v>
       </c>
       <c r="B193" t="n">
-        <v>1494.785</v>
+        <v>746.293</v>
       </c>
       <c r="C193" t="n">
-        <v>413</v>
+        <v>405</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>1494.852</v>
+        <v>746.326</v>
       </c>
       <c r="B194" t="n">
-        <v>1495.485</v>
+        <v>748.293</v>
       </c>
       <c r="C194" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>1495.552</v>
+        <v>748.326</v>
       </c>
       <c r="B195" t="n">
-        <v>1496.285</v>
+        <v>749.293</v>
       </c>
       <c r="C195" t="n">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>1496.318</v>
+        <v>749.326</v>
       </c>
       <c r="B196" t="n">
-        <v>1497.252</v>
+        <v>750.759</v>
       </c>
       <c r="C196" t="n">
-        <v>404</v>
+        <v>413</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>1497.352</v>
+        <v>750.792</v>
       </c>
       <c r="B197" t="n">
-        <v>1497.585</v>
+        <v>751.492</v>
       </c>
       <c r="C197" t="n">
         <v>412</v>
@@ -2591,10 +2591,10 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>1497.652</v>
+        <v>753.426</v>
       </c>
       <c r="B198" t="n">
-        <v>1498.085</v>
+        <v>753.9589999999999</v>
       </c>
       <c r="C198" t="n">
         <v>405</v>
@@ -2602,197 +2602,197 @@
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>1498.252</v>
+        <v>753.992</v>
       </c>
       <c r="B199" t="n">
-        <v>1499.185</v>
+        <v>755.226</v>
       </c>
       <c r="C199" t="n">
-        <v>406</v>
+        <v>413</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>1499.385</v>
+        <v>755.259</v>
       </c>
       <c r="B200" t="n">
-        <v>1500.385</v>
+        <v>756.592</v>
       </c>
       <c r="C200" t="n">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>1509.118</v>
+        <v>756.626</v>
       </c>
       <c r="B201" t="n">
-        <v>1510.218</v>
+        <v>757.992</v>
       </c>
       <c r="C201" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>1510.285</v>
+        <v>758.026</v>
       </c>
       <c r="B202" t="n">
-        <v>1511.885</v>
+        <v>758.992</v>
       </c>
       <c r="C202" t="n">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>1513.785</v>
+        <v>760.259</v>
       </c>
       <c r="B203" t="n">
-        <v>1513.985</v>
+        <v>761.092</v>
       </c>
       <c r="C203" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>1518.318</v>
+        <v>761.126</v>
       </c>
       <c r="B204" t="n">
-        <v>1518.785</v>
+        <v>763.3920000000001</v>
       </c>
       <c r="C204" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>1518.818</v>
+        <v>763.426</v>
       </c>
       <c r="B205" t="n">
-        <v>1520.985</v>
+        <v>765.292</v>
       </c>
       <c r="C205" t="n">
-        <v>404</v>
+        <v>409</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>1521.051</v>
+        <v>765.326</v>
       </c>
       <c r="B206" t="n">
-        <v>1521.985</v>
+        <v>766.792</v>
       </c>
       <c r="C206" t="n">
-        <v>412</v>
+        <v>413</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>1535.918</v>
+        <v>766.826</v>
       </c>
       <c r="B207" t="n">
-        <v>1536.651</v>
+        <v>768.559</v>
       </c>
       <c r="C207" t="n">
-        <v>405</v>
+        <v>412</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>1536.751</v>
+        <v>770.126</v>
       </c>
       <c r="B208" t="n">
-        <v>1542.551</v>
+        <v>771.059</v>
       </c>
       <c r="C208" t="n">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>1548.485</v>
+        <v>771.092</v>
       </c>
       <c r="B209" t="n">
-        <v>1549.185</v>
+        <v>772.859</v>
       </c>
       <c r="C209" t="n">
-        <v>408</v>
+        <v>413</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>1549.251</v>
+        <v>772.8920000000001</v>
       </c>
       <c r="B210" t="n">
-        <v>1550.084</v>
+        <v>774.192</v>
       </c>
       <c r="C210" t="n">
-        <v>412</v>
+        <v>407</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>1567.784</v>
+        <v>774.226</v>
       </c>
       <c r="B211" t="n">
-        <v>1568.884</v>
+        <v>775.792</v>
       </c>
       <c r="C211" t="n">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>1568.918</v>
+        <v>775.826</v>
       </c>
       <c r="B212" t="n">
-        <v>1570.984</v>
+        <v>776.092</v>
       </c>
       <c r="C212" t="n">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>1571.618</v>
+        <v>776.126</v>
       </c>
       <c r="B213" t="n">
-        <v>1572.118</v>
+        <v>781.192</v>
       </c>
       <c r="C213" t="n">
-        <v>412</v>
+        <v>405</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>1574.618</v>
+        <v>781.226</v>
       </c>
       <c r="B214" t="n">
-        <v>1575.384</v>
+        <v>783.8920000000001</v>
       </c>
       <c r="C214" t="n">
-        <v>405</v>
+        <v>409</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>1575.451</v>
+        <v>783.925</v>
       </c>
       <c r="B215" t="n">
-        <v>1577.284</v>
+        <v>784.8920000000001</v>
       </c>
       <c r="C215" t="n">
-        <v>404</v>
+        <v>413</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>1579.118</v>
+        <v>784.925</v>
       </c>
       <c r="B216" t="n">
-        <v>1579.884</v>
+        <v>785.825</v>
       </c>
       <c r="C216" t="n">
         <v>412</v>
@@ -2800,10 +2800,10 @@
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>1583.717</v>
+        <v>789.592</v>
       </c>
       <c r="B217" t="n">
-        <v>1584.584</v>
+        <v>790.3920000000001</v>
       </c>
       <c r="C217" t="n">
         <v>405</v>
@@ -2811,13 +2811,794 @@
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>1584.651</v>
+        <v>790.425</v>
       </c>
       <c r="B218" t="n">
-        <v>1588.951</v>
+        <v>791.792</v>
       </c>
       <c r="C218" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>791.825</v>
+      </c>
+      <c r="B219" t="n">
+        <v>792.792</v>
+      </c>
+      <c r="C219" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>792.825</v>
+      </c>
+      <c r="B220" t="n">
+        <v>793.8920000000001</v>
+      </c>
+      <c r="C220" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>793.925</v>
+      </c>
+      <c r="B221" t="n">
+        <v>794.8920000000001</v>
+      </c>
+      <c r="C221" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>797.825</v>
+      </c>
+      <c r="B222" t="n">
+        <v>798.759</v>
+      </c>
+      <c r="C222" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>798.792</v>
+      </c>
+      <c r="B223" t="n">
+        <v>799.859</v>
+      </c>
+      <c r="C223" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>799.8920000000001</v>
+      </c>
+      <c r="B224" t="n">
+        <v>800.592</v>
+      </c>
+      <c r="C224" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>800.625</v>
+      </c>
+      <c r="B225" t="n">
+        <v>801.792</v>
+      </c>
+      <c r="C225" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>801.825</v>
+      </c>
+      <c r="B226" t="n">
+        <v>802.925</v>
+      </c>
+      <c r="C226" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>805.925</v>
+      </c>
+      <c r="B227" t="n">
+        <v>806.925</v>
+      </c>
+      <c r="C227" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>806.9589999999999</v>
+      </c>
+      <c r="B228" t="n">
+        <v>808.292</v>
+      </c>
+      <c r="C228" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>808.325</v>
+      </c>
+      <c r="B229" t="n">
+        <v>809.825</v>
+      </c>
+      <c r="C229" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>809.859</v>
+      </c>
+      <c r="B230" t="n">
+        <v>810.8920000000001</v>
+      </c>
+      <c r="C230" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>810.925</v>
+      </c>
+      <c r="B231" t="n">
+        <v>811.592</v>
+      </c>
+      <c r="C231" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>813.825</v>
+      </c>
+      <c r="B232" t="n">
+        <v>815.192</v>
+      </c>
+      <c r="C232" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>815.225</v>
+      </c>
+      <c r="B233" t="n">
+        <v>816.292</v>
+      </c>
+      <c r="C233" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>816.325</v>
+      </c>
+      <c r="B234" t="n">
+        <v>817.192</v>
+      </c>
+      <c r="C234" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>817.225</v>
+      </c>
+      <c r="B235" t="n">
+        <v>818.192</v>
+      </c>
+      <c r="C235" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>818.225</v>
+      </c>
+      <c r="B236" t="n">
+        <v>819.092</v>
+      </c>
+      <c r="C236" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>821.325</v>
+      </c>
+      <c r="B237" t="n">
+        <v>822.092</v>
+      </c>
+      <c r="C237" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>822.125</v>
+      </c>
+      <c r="B238" t="n">
+        <v>823.158</v>
+      </c>
+      <c r="C238" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>823.192</v>
+      </c>
+      <c r="B239" t="n">
+        <v>824.292</v>
+      </c>
+      <c r="C239" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>824.325</v>
+      </c>
+      <c r="B240" t="n">
+        <v>825.325</v>
+      </c>
+      <c r="C240" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>825.3920000000001</v>
+      </c>
+      <c r="B241" t="n">
+        <v>826.258</v>
+      </c>
+      <c r="C241" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>835.092</v>
+      </c>
+      <c r="B242" t="n">
+        <v>849.125</v>
+      </c>
+      <c r="C242" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>849.158</v>
+      </c>
+      <c r="B243" t="n">
+        <v>849.758</v>
+      </c>
+      <c r="C243" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>855.625</v>
+      </c>
+      <c r="B244" t="n">
+        <v>859.7910000000001</v>
+      </c>
+      <c r="C244" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>859.925</v>
+      </c>
+      <c r="B245" t="n">
+        <v>860.391</v>
+      </c>
+      <c r="C245" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>860.425</v>
+      </c>
+      <c r="B246" t="n">
+        <v>863.691</v>
+      </c>
+      <c r="C246" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>863.725</v>
+      </c>
+      <c r="B247" t="n">
+        <v>864.458</v>
+      </c>
+      <c r="C247" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>864.491</v>
+      </c>
+      <c r="B248" t="n">
+        <v>865.958</v>
+      </c>
+      <c r="C248" t="n">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>865.991</v>
+      </c>
+      <c r="B249" t="n">
+        <v>866.525</v>
+      </c>
+      <c r="C249" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>866.558</v>
+      </c>
+      <c r="B250" t="n">
+        <v>873.258</v>
+      </c>
+      <c r="C250" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>873.2910000000001</v>
+      </c>
+      <c r="B251" t="n">
+        <v>873.7910000000001</v>
+      </c>
+      <c r="C251" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>880.958</v>
+      </c>
+      <c r="B252" t="n">
+        <v>891.7910000000001</v>
+      </c>
+      <c r="C252" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>891.824</v>
+      </c>
+      <c r="B253" t="n">
+        <v>892.891</v>
+      </c>
+      <c r="C253" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>898.224</v>
+      </c>
+      <c r="B254" t="n">
+        <v>899.391</v>
+      </c>
+      <c r="C254" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>899.424</v>
+      </c>
+      <c r="B255" t="n">
+        <v>905.824</v>
+      </c>
+      <c r="C255" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>905.8579999999999</v>
+      </c>
+      <c r="B256" t="n">
+        <v>906.491</v>
+      </c>
+      <c r="C256" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>914.224</v>
+      </c>
+      <c r="B257" t="n">
+        <v>914.8579999999999</v>
+      </c>
+      <c r="C257" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>914.891</v>
+      </c>
+      <c r="B258" t="n">
+        <v>917.124</v>
+      </c>
+      <c r="C258" t="n">
         <v>404</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>917.157</v>
+      </c>
+      <c r="B259" t="n">
+        <v>917.857</v>
+      </c>
+      <c r="C259" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>920.324</v>
+      </c>
+      <c r="B260" t="n">
+        <v>921.091</v>
+      </c>
+      <c r="C260" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>921.124</v>
+      </c>
+      <c r="B261" t="n">
+        <v>923.2910000000001</v>
+      </c>
+      <c r="C261" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>923.324</v>
+      </c>
+      <c r="B262" t="n">
+        <v>923.991</v>
+      </c>
+      <c r="C262" t="n">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>924.024</v>
+      </c>
+      <c r="B263" t="n">
+        <v>924.991</v>
+      </c>
+      <c r="C263" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>929.024</v>
+      </c>
+      <c r="B264" t="n">
+        <v>930.2569999999999</v>
+      </c>
+      <c r="C264" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>930.324</v>
+      </c>
+      <c r="B265" t="n">
+        <v>937.2569999999999</v>
+      </c>
+      <c r="C265" t="n">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>938.124</v>
+      </c>
+      <c r="B266" t="n">
+        <v>939.7569999999999</v>
+      </c>
+      <c r="C266" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>939.7910000000001</v>
+      </c>
+      <c r="B267" t="n">
+        <v>941.124</v>
+      </c>
+      <c r="C267" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>945.024</v>
+      </c>
+      <c r="B268" t="n">
+        <v>946.224</v>
+      </c>
+      <c r="C268" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>946.2910000000001</v>
+      </c>
+      <c r="B269" t="n">
+        <v>947.091</v>
+      </c>
+      <c r="C269" t="n">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>947.124</v>
+      </c>
+      <c r="B270" t="n">
+        <v>948.191</v>
+      </c>
+      <c r="C270" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>948.224</v>
+      </c>
+      <c r="B271" t="n">
+        <v>949.391</v>
+      </c>
+      <c r="C271" t="n">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>949.424</v>
+      </c>
+      <c r="B272" t="n">
+        <v>950.99</v>
+      </c>
+      <c r="C272" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>954.724</v>
+      </c>
+      <c r="B273" t="n">
+        <v>955.7569999999999</v>
+      </c>
+      <c r="C273" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>955.79</v>
+      </c>
+      <c r="B274" t="n">
+        <v>956.09</v>
+      </c>
+      <c r="C274" t="n">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>956.124</v>
+      </c>
+      <c r="B275" t="n">
+        <v>958.79</v>
+      </c>
+      <c r="C275" t="n">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>958.824</v>
+      </c>
+      <c r="B276" t="n">
+        <v>959.657</v>
+      </c>
+      <c r="C276" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>968.324</v>
+      </c>
+      <c r="B277" t="n">
+        <v>968.89</v>
+      </c>
+      <c r="C277" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>968.924</v>
+      </c>
+      <c r="B278" t="n">
+        <v>975.49</v>
+      </c>
+      <c r="C278" t="n">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>975.524</v>
+      </c>
+      <c r="B279" t="n">
+        <v>976.1900000000001</v>
+      </c>
+      <c r="C279" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>985.59</v>
+      </c>
+      <c r="B280" t="n">
+        <v>986.29</v>
+      </c>
+      <c r="C280" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>986.323</v>
+      </c>
+      <c r="B281" t="n">
+        <v>986.89</v>
+      </c>
+      <c r="C281" t="n">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>986.923</v>
+      </c>
+      <c r="B282" t="n">
+        <v>988.323</v>
+      </c>
+      <c r="C282" t="n">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>989.423</v>
+      </c>
+      <c r="B283" t="n">
+        <v>989.99</v>
+      </c>
+      <c r="C283" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>993.123</v>
+      </c>
+      <c r="B284" t="n">
+        <v>993.89</v>
+      </c>
+      <c r="C284" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>993.923</v>
+      </c>
+      <c r="B285" t="n">
+        <v>996.023</v>
+      </c>
+      <c r="C285" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>996.057</v>
+      </c>
+      <c r="B286" t="n">
+        <v>996.557</v>
+      </c>
+      <c r="C286" t="n">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>996.59</v>
+      </c>
+      <c r="B287" t="n">
+        <v>997.99</v>
+      </c>
+      <c r="C287" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>1002.523</v>
+      </c>
+      <c r="B288" t="n">
+        <v>1003.49</v>
+      </c>
+      <c r="C288" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>1003.523</v>
+      </c>
+      <c r="B289" t="n">
+        <v>1005.69</v>
+      </c>
+      <c r="C289" t="n">
+        <v>412</v>
       </c>
     </row>
   </sheetData>

</xml_diff>